<commit_message>
chore: fix Предметы.xlsx data (integer damage/defense, trim item names)
</commit_message>
<xml_diff>
--- a/RPGO.Editor/Resources/Предметы.xlsx
+++ b/RPGO.Editor/Resources/Предметы.xlsx
@@ -136,22 +136,22 @@
     <t>Меч капитана</t>
   </si>
   <si>
-    <t xml:space="preserve">	Меч генерала</t>
+    <t xml:space="preserve">Меч генерала</t>
   </si>
   <si>
-    <t xml:space="preserve">	Меч маршала</t>
+    <t xml:space="preserve">Меч маршала</t>
   </si>
   <si>
-    <t xml:space="preserve">	Меч герцога</t>
+    <t xml:space="preserve">Меч герцога</t>
   </si>
   <si>
-    <t xml:space="preserve">	Меч короля</t>
+    <t xml:space="preserve">Меч короля</t>
   </si>
   <si>
     <t>Меч императора</t>
   </si>
   <si>
-    <t xml:space="preserve">	Клинок Легенды</t>
+    <t xml:space="preserve">Клинок Легенды</t>
   </si>
   <si>
     <t>Меч лейтенанта</t>
@@ -196,16 +196,16 @@
     <t>Топор новичка</t>
   </si>
   <si>
-    <t xml:space="preserve">	Топор охотника</t>
+    <t xml:space="preserve">Топор охотника</t>
   </si>
   <si>
-    <t xml:space="preserve">	Топор берсерка</t>
+    <t xml:space="preserve">Топор берсерка</t>
   </si>
   <si>
     <t>Волчий топор</t>
   </si>
   <si>
-    <t xml:space="preserve">	Топор медведя</t>
+    <t xml:space="preserve">Топор медведя</t>
   </si>
   <si>
     <t>Топор ястреба</t>
@@ -214,13 +214,13 @@
     <t>Топор дракона</t>
   </si>
   <si>
-    <t xml:space="preserve">	Топор великана</t>
+    <t xml:space="preserve">Топор великана</t>
   </si>
   <si>
     <t>Топор титана</t>
   </si>
   <si>
-    <t xml:space="preserve">	Топор бога</t>
+    <t xml:space="preserve">Топор бога</t>
   </si>
   <si>
     <t>Кромсатель Небес</t>
@@ -241,25 +241,25 @@
     <t>Булава правосудия</t>
   </si>
   <si>
-    <t xml:space="preserve">	Булава инквизитора</t>
+    <t xml:space="preserve">Булава инквизитора</t>
   </si>
   <si>
     <t>Палица крестоносца</t>
   </si>
   <si>
-    <t xml:space="preserve">	Дубина епископа</t>
+    <t xml:space="preserve">Дубина епископа</t>
   </si>
   <si>
-    <t xml:space="preserve">	Булава архиепископа</t>
+    <t xml:space="preserve">Булава архиепископа</t>
   </si>
   <si>
     <t>Палица Собора</t>
   </si>
   <si>
-    <t xml:space="preserve">	Длань Святого</t>
+    <t xml:space="preserve">Длань Святого</t>
   </si>
   <si>
-    <t xml:space="preserve">	Длань Судьи</t>
+    <t xml:space="preserve">Длань Судьи</t>
   </si>
   <si>
     <t>Молот</t>
@@ -268,34 +268,34 @@
     <t>Кузнечный молот</t>
   </si>
   <si>
-    <t xml:space="preserve">	Боевой молот</t>
+    <t xml:space="preserve">Боевой молот</t>
   </si>
   <si>
-    <t xml:space="preserve">	Молот горных недр</t>
+    <t xml:space="preserve">Молот горных недр</t>
   </si>
   <si>
-    <t xml:space="preserve">	Тяжелый молот</t>
+    <t xml:space="preserve">Тяжелый молот</t>
   </si>
   <si>
-    <t xml:space="preserve">	Дробящий молот</t>
+    <t xml:space="preserve">Дробящий молот</t>
   </si>
   <si>
     <t xml:space="preserve">	Молот великанов</t>
   </si>
   <si>
-    <t xml:space="preserve">	Кузня грома</t>
+    <t xml:space="preserve">Кузня грома</t>
   </si>
   <si>
-    <t xml:space="preserve">	Молот разлома</t>
+    <t xml:space="preserve">Молот разлома</t>
   </si>
   <si>
-    <t xml:space="preserve">	Длань титана</t>
+    <t xml:space="preserve">Длань титана</t>
   </si>
   <si>
     <t xml:space="preserve">	Громовой молот</t>
   </si>
   <si>
-    <t xml:space="preserve">	Молот Мироздания</t>
+    <t xml:space="preserve">Молот Мироздания</t>
   </si>
   <si>
     <t>Кинжал</t>
@@ -304,34 +304,34 @@
     <t>Кухонный нож</t>
   </si>
   <si>
-    <t xml:space="preserve">	Кинжал разведчика</t>
+    <t xml:space="preserve">Кинжал разведчика</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лезвие ночи</t>
+    <t xml:space="preserve">Лезвие ночи</t>
   </si>
   <si>
-    <t xml:space="preserve">	Шепот смерти</t>
+    <t xml:space="preserve">Шепот смерти</t>
   </si>
   <si>
     <t>Клык тени</t>
   </si>
   <si>
-    <t xml:space="preserve">	Кинжал призрака</t>
+    <t xml:space="preserve">Кинжал призрака</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лезвие тумана</t>
+    <t xml:space="preserve">Лезвие тумана</t>
   </si>
   <si>
-    <t xml:space="preserve">	Укус скорпиона</t>
+    <t xml:space="preserve">Укус скорпиона</t>
   </si>
   <si>
-    <t xml:space="preserve">	Кинжал тьмы</t>
+    <t xml:space="preserve">Кинжал тьмы</t>
   </si>
   <si>
-    <t xml:space="preserve">	Жало смерти</t>
+    <t xml:space="preserve">Жало смерти</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лезвие Вечности</t>
+    <t xml:space="preserve">Лезвие Вечности</t>
   </si>
   <si>
     <t>Гримуар</t>
@@ -343,7 +343,7 @@
     <t>Гримуар послушника</t>
   </si>
   <si>
-    <t xml:space="preserve">	Книга стихий</t>
+    <t xml:space="preserve">Книга стихий</t>
   </si>
   <si>
     <t>Книга тайн</t>
@@ -355,19 +355,19 @@
     <t>Гримуар древних</t>
   </si>
   <si>
-    <t xml:space="preserve">	Книга теней</t>
+    <t xml:space="preserve">Книга теней</t>
   </si>
   <si>
-    <t xml:space="preserve">	Гримуар бессмертных</t>
+    <t xml:space="preserve">Гримуар бессмертных</t>
   </si>
   <si>
-    <t xml:space="preserve">	Книга хаоса</t>
+    <t xml:space="preserve">Книга хаоса</t>
   </si>
   <si>
-    <t xml:space="preserve">	Гримуар бездны</t>
+    <t xml:space="preserve">Гримуар бездны</t>
   </si>
   <si>
-    <t xml:space="preserve">	Кодекс Мироздания</t>
+    <t xml:space="preserve">Кодекс Мироздания</t>
   </si>
   <si>
     <t>Левая рука</t>
@@ -376,37 +376,37 @@
     <t>Сфера</t>
   </si>
   <si>
-    <t xml:space="preserve">	Грязный кристалл</t>
+    <t xml:space="preserve">Грязный кристалл</t>
   </si>
   <si>
-    <t xml:space="preserve">	Сфера послушника</t>
+    <t xml:space="preserve">Сфера послушника</t>
   </si>
   <si>
     <t>Огненная сфера</t>
   </si>
   <si>
-    <t xml:space="preserve">	Ледяной шар</t>
+    <t xml:space="preserve">Ледяной шар</t>
   </si>
   <si>
-    <t xml:space="preserve">	Сфера бурь</t>
+    <t xml:space="preserve">Сфера бурь</t>
   </si>
   <si>
-    <t xml:space="preserve">	Звездный шар</t>
+    <t xml:space="preserve">Звездный шар</t>
   </si>
   <si>
-    <t xml:space="preserve">	Сфера порталов</t>
+    <t xml:space="preserve">Сфера порталов</t>
   </si>
   <si>
-    <t xml:space="preserve">	Шар света</t>
+    <t xml:space="preserve">Шар света</t>
   </si>
   <si>
-    <t xml:space="preserve">	Сфера тьмы</t>
+    <t xml:space="preserve">Сфера тьмы</t>
   </si>
   <si>
-    <t xml:space="preserve">	Око хаоса</t>
+    <t xml:space="preserve">Око хаоса</t>
   </si>
   <si>
-    <t xml:space="preserve">	Сердце Вселенной</t>
+    <t xml:space="preserve">Сердце Вселенной</t>
   </si>
   <si>
     <t>Двуручный</t>
@@ -415,37 +415,37 @@
     <t>Лук</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лук крестьянина</t>
+    <t xml:space="preserve">Лук крестьянина</t>
   </si>
   <si>
     <t>Лук охотника</t>
   </si>
   <si>
-    <t xml:space="preserve">	Длинный лук</t>
+    <t xml:space="preserve">Длинный лук</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лук скаута</t>
+    <t xml:space="preserve">Лук скаута</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лук ветра</t>
+    <t xml:space="preserve">Лук ветра</t>
   </si>
   <si>
     <t>Лук ястреба</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лук дракона</t>
+    <t xml:space="preserve">Лук дракона</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лук бури</t>
+    <t xml:space="preserve">Лук бури</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лук теней</t>
+    <t xml:space="preserve">Лук теней</t>
   </si>
   <si>
-    <t xml:space="preserve">	Лук возмездия</t>
+    <t xml:space="preserve">Лук возмездия</t>
   </si>
   <si>
-    <t xml:space="preserve">	Шепот Вечности</t>
+    <t xml:space="preserve">Шепот Вечности</t>
   </si>
   <si>
     <t>Посох</t>
@@ -454,70 +454,70 @@
     <t>Посох ученика</t>
   </si>
   <si>
-    <t xml:space="preserve">	Посох мага</t>
+    <t xml:space="preserve">Посох мага</t>
   </si>
   <si>
     <t>Посох стихий</t>
   </si>
   <si>
-    <t xml:space="preserve">	Посох судьбы</t>
+    <t xml:space="preserve">Посох судьбы</t>
   </si>
   <si>
     <t>Посох времени</t>
   </si>
   <si>
-    <t xml:space="preserve">	Посох драконьего сердца</t>
+    <t xml:space="preserve">Посох драконьего сердца</t>
   </si>
   <si>
-    <t xml:space="preserve">	Посох бессмертных</t>
+    <t xml:space="preserve">Посох бессмертных</t>
   </si>
   <si>
     <t>Посох хаоса</t>
   </si>
   <si>
-    <t xml:space="preserve">	Посох бездны</t>
+    <t xml:space="preserve">Посох бездны</t>
   </si>
   <si>
-    <t xml:space="preserve">	Посох творения</t>
+    <t xml:space="preserve">Посох творения</t>
   </si>
   <si>
-    <t xml:space="preserve">	Ось Мироздания</t>
+    <t xml:space="preserve">Ось Мироздания</t>
   </si>
   <si>
     <t>Большой меч</t>
   </si>
   <si>
-    <t xml:space="preserve">	Двуручный меч</t>
+    <t xml:space="preserve">Двуручный меч</t>
   </si>
   <si>
     <t>Гладкий двуручный меч</t>
   </si>
   <si>
-    <t xml:space="preserve">	Палаш</t>
+    <t xml:space="preserve">Палаш</t>
   </si>
   <si>
-    <t xml:space="preserve">	Длинный меч</t>
+    <t xml:space="preserve">Длинный меч</t>
   </si>
   <si>
-    <t xml:space="preserve">	Клинок героя</t>
+    <t xml:space="preserve">Клинок героя</t>
   </si>
   <si>
-    <t xml:space="preserve">	Клинок паладина</t>
+    <t xml:space="preserve">Клинок паладина</t>
   </si>
   <si>
-    <t xml:space="preserve">	Клинок короля</t>
+    <t xml:space="preserve">Клинок короля</t>
   </si>
   <si>
-    <t xml:space="preserve">	Клинок великана</t>
+    <t xml:space="preserve">Клинок великана</t>
   </si>
   <si>
-    <t xml:space="preserve">	Клинок титана</t>
+    <t xml:space="preserve">Клинок титана</t>
   </si>
   <si>
     <t>Рассекатель гор</t>
   </si>
   <si>
-    <t xml:space="preserve">	Клинок Армагеддона</t>
+    <t xml:space="preserve">Клинок Армагеддона</t>
   </si>
   <si>
     <t>Секира</t>
@@ -526,34 +526,34 @@
     <t>Секира новобранца</t>
   </si>
   <si>
-    <t xml:space="preserve">	Боевая секира</t>
+    <t xml:space="preserve">Боевая секира</t>
   </si>
   <si>
-    <t xml:space="preserve">	Секира палача</t>
+    <t xml:space="preserve">Секира палача</t>
   </si>
   <si>
-    <t xml:space="preserve">	Секира отчаяния</t>
+    <t xml:space="preserve">Секира отчаяния</t>
   </si>
   <si>
-    <t xml:space="preserve">	Секира смерти</t>
+    <t xml:space="preserve">Секира смерти</t>
   </si>
   <si>
-    <t xml:space="preserve">	Секира ужаса</t>
+    <t xml:space="preserve">Секира ужаса</t>
   </si>
   <si>
-    <t xml:space="preserve">	Секира мясника</t>
+    <t xml:space="preserve">Секира мясника</t>
   </si>
   <si>
-    <t xml:space="preserve">	Секира истребления</t>
+    <t xml:space="preserve">Секира истребления</t>
   </si>
   <si>
-    <t xml:space="preserve">	Секира катастрофы</t>
+    <t xml:space="preserve">Секира катастрофы</t>
   </si>
   <si>
-    <t xml:space="preserve">	Секира апокалипсиса</t>
+    <t xml:space="preserve">Секира апокалипсиса</t>
   </si>
   <si>
-    <t xml:space="preserve">	Кромсатель Миров</t>
+    <t xml:space="preserve">Кромсатель Миров</t>
   </si>
   <si>
     <t>Алебарда</t>
@@ -562,88 +562,88 @@
     <t>Алебарда новобранца</t>
   </si>
   <si>
-    <t xml:space="preserve">	Алебарда стражи</t>
+    <t xml:space="preserve">Алебарда стражи</t>
   </si>
   <si>
-    <t xml:space="preserve">	Алебарда пехотинца</t>
+    <t xml:space="preserve">Алебарда пехотинца</t>
   </si>
   <si>
-    <t xml:space="preserve">	Алебарда легионера</t>
+    <t xml:space="preserve">Алебарда легионера</t>
   </si>
   <si>
-    <t xml:space="preserve">	Алебарда защиты</t>
+    <t xml:space="preserve">Алебарда защиты</t>
   </si>
   <si>
-    <t xml:space="preserve">	Алебарда стен</t>
+    <t xml:space="preserve">Алебарда стен</t>
   </si>
   <si>
-    <t xml:space="preserve">	Алебарда крепости</t>
+    <t xml:space="preserve">Алебарда крепости</t>
   </si>
   <si>
-    <t xml:space="preserve">	Алебарда героя</t>
+    <t xml:space="preserve">Алебарда героя</t>
   </si>
   <si>
     <t>Алебарда империи</t>
   </si>
   <si>
-    <t xml:space="preserve">	Алебарда судьбы</t>
+    <t xml:space="preserve">Алебарда судьбы</t>
   </si>
   <si>
     <t>Копье</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье крестьянина</t>
+    <t xml:space="preserve">Копье крестьянина</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье охотника</t>
+    <t xml:space="preserve">Копье охотника</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье воина</t>
+    <t xml:space="preserve">Копье воина</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье бронебойное</t>
+    <t xml:space="preserve">Копье бронебойное</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье дракона</t>
+    <t xml:space="preserve">Копье дракона</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье молнии</t>
+    <t xml:space="preserve">Копье молнии</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье великана</t>
+    <t xml:space="preserve">Копье великана</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье грозы</t>
+    <t xml:space="preserve">Копье грозы</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье титана</t>
+    <t xml:space="preserve">Копье титана</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье судьбы</t>
+    <t xml:space="preserve">Копье судьбы</t>
   </si>
   <si>
-    <t xml:space="preserve">	Копье Армагеддона</t>
+    <t xml:space="preserve">Копье Армагеддона</t>
   </si>
   <si>
     <t>Большой молот</t>
   </si>
   <si>
-    <t xml:space="preserve">	Молот силача</t>
+    <t xml:space="preserve">Молот силача</t>
   </si>
   <si>
     <t>Боевой молот</t>
   </si>
   <si>
-    <t xml:space="preserve">	Молот грома</t>
+    <t xml:space="preserve">Молот грома</t>
   </si>
   <si>
-    <t xml:space="preserve">	Молот землетрясения</t>
+    <t xml:space="preserve">Молот землетрясения</t>
   </si>
   <si>
-    <t xml:space="preserve">	Молот сокрушения</t>
+    <t xml:space="preserve">Молот сокрушения</t>
   </si>
   <si>
-    <t xml:space="preserve">	Молот Сотворения</t>
+    <t xml:space="preserve">Молот Сотворения</t>
   </si>
   <si>
     <t>Щит</t>
@@ -652,34 +652,34 @@
     <t>Деревянный щит</t>
   </si>
   <si>
-    <t xml:space="preserve">	Щит стража</t>
+    <t xml:space="preserve">Щит стража</t>
   </si>
   <si>
-    <t xml:space="preserve">	Щит пехотинца</t>
+    <t xml:space="preserve">Щит пехотинца</t>
   </si>
   <si>
-    <t xml:space="preserve">	Щит легионера</t>
+    <t xml:space="preserve">Щит легионера</t>
   </si>
   <si>
-    <t xml:space="preserve">	Щит капитана</t>
+    <t xml:space="preserve">Щит капитана</t>
   </si>
   <si>
-    <t xml:space="preserve">	Щит генерала</t>
+    <t xml:space="preserve">Щит генерала</t>
   </si>
   <si>
-    <t xml:space="preserve">	Щит маршала</t>
+    <t xml:space="preserve">Щит маршала</t>
   </si>
   <si>
-    <t xml:space="preserve">	Щит герцога</t>
+    <t xml:space="preserve">Щит герцога</t>
   </si>
   <si>
-    <t xml:space="preserve">	Щит короля</t>
+    <t xml:space="preserve">Щит короля</t>
   </si>
   <si>
-    <t xml:space="preserve">	Щит императора</t>
+    <t xml:space="preserve">Щит императора</t>
   </si>
   <si>
-    <t xml:space="preserve">	Эгида Легиона</t>
+    <t xml:space="preserve">Эгида Легиона</t>
   </si>
   <si>
     <t>Диапозон бонусов</t>
@@ -700,7 +700,7 @@
     <t>Длань титана</t>
   </si>
   <si>
-    <t xml:space="preserve">	Молот гнева</t>
+    <t xml:space="preserve">Молот гнева</t>
   </si>
   <si>
     <t>Алебарда разлома</t>
@@ -1461,7 +1461,7 @@
         <v>26</v>
       </c>
       <c r="G5" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>21</v>
@@ -1502,7 +1502,7 @@
         <v>27</v>
       </c>
       <c r="G6" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>21</v>
@@ -1543,7 +1543,7 @@
         <v>28</v>
       </c>
       <c r="G7" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>21</v>
@@ -1637,7 +1637,7 @@
         <v>26</v>
       </c>
       <c r="G9" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>21</v>
@@ -1678,7 +1678,7 @@
         <v>27</v>
       </c>
       <c r="G10" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>21</v>
@@ -1719,7 +1719,7 @@
         <v>28</v>
       </c>
       <c r="G11" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>21</v>
@@ -1813,7 +1813,7 @@
         <v>26</v>
       </c>
       <c r="G13" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>21</v>
@@ -1854,7 +1854,7 @@
         <v>27</v>
       </c>
       <c r="G14" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>21</v>
@@ -1895,7 +1895,7 @@
         <v>28</v>
       </c>
       <c r="G15" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>21</v>
@@ -1989,7 +1989,7 @@
         <v>26</v>
       </c>
       <c r="G17" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>21</v>
@@ -2030,7 +2030,7 @@
         <v>27</v>
       </c>
       <c r="G18" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>21</v>
@@ -2071,7 +2071,7 @@
         <v>28</v>
       </c>
       <c r="G19" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>21</v>
@@ -2165,7 +2165,7 @@
         <v>26</v>
       </c>
       <c r="G21" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>21</v>
@@ -2206,7 +2206,7 @@
         <v>27</v>
       </c>
       <c r="G22" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>21</v>
@@ -2247,7 +2247,7 @@
         <v>28</v>
       </c>
       <c r="G23" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>21</v>
@@ -2341,7 +2341,7 @@
         <v>26</v>
       </c>
       <c r="G25" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>21</v>
@@ -2382,7 +2382,7 @@
         <v>27</v>
       </c>
       <c r="G26" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>21</v>
@@ -2423,7 +2423,7 @@
         <v>28</v>
       </c>
       <c r="G27" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>21</v>
@@ -2517,7 +2517,7 @@
         <v>26</v>
       </c>
       <c r="G29" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>21</v>
@@ -2558,7 +2558,7 @@
         <v>27</v>
       </c>
       <c r="G30" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>21</v>
@@ -2599,7 +2599,7 @@
         <v>28</v>
       </c>
       <c r="G31" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H31" s="6" t="s">
         <v>21</v>
@@ -2693,7 +2693,7 @@
         <v>26</v>
       </c>
       <c r="G33" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>21</v>
@@ -2734,7 +2734,7 @@
         <v>27</v>
       </c>
       <c r="G34" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H34" s="6" t="s">
         <v>21</v>
@@ -2775,7 +2775,7 @@
         <v>28</v>
       </c>
       <c r="G35" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H35" s="6" t="s">
         <v>21</v>
@@ -2869,7 +2869,7 @@
         <v>26</v>
       </c>
       <c r="G37" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>21</v>
@@ -2910,7 +2910,7 @@
         <v>27</v>
       </c>
       <c r="G38" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>21</v>
@@ -2951,7 +2951,7 @@
         <v>28</v>
       </c>
       <c r="G39" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>21</v>
@@ -3045,7 +3045,7 @@
         <v>26</v>
       </c>
       <c r="G41" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>21</v>
@@ -3086,7 +3086,7 @@
         <v>27</v>
       </c>
       <c r="G42" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H42" s="6" t="s">
         <v>21</v>
@@ -3127,7 +3127,7 @@
         <v>28</v>
       </c>
       <c r="G43" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>21</v>
@@ -3274,7 +3274,7 @@
         <v>26</v>
       </c>
       <c r="G46" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H46" s="6" t="s">
         <v>21</v>
@@ -3315,7 +3315,7 @@
         <v>27</v>
       </c>
       <c r="G47" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H47" s="6" t="s">
         <v>21</v>
@@ -3356,7 +3356,7 @@
         <v>28</v>
       </c>
       <c r="G48" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H48" s="6" t="s">
         <v>21</v>
@@ -3450,7 +3450,7 @@
         <v>26</v>
       </c>
       <c r="G50" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H50" s="6" t="s">
         <v>21</v>
@@ -3491,7 +3491,7 @@
         <v>27</v>
       </c>
       <c r="G51" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H51" s="6" t="s">
         <v>21</v>
@@ -3532,7 +3532,7 @@
         <v>28</v>
       </c>
       <c r="G52" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>21</v>
@@ -3626,7 +3626,7 @@
         <v>26</v>
       </c>
       <c r="G54" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H54" s="6" t="s">
         <v>21</v>
@@ -3667,7 +3667,7 @@
         <v>27</v>
       </c>
       <c r="G55" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H55" s="6" t="s">
         <v>21</v>
@@ -3708,7 +3708,7 @@
         <v>28</v>
       </c>
       <c r="G56" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H56" s="6" t="s">
         <v>21</v>
@@ -3802,7 +3802,7 @@
         <v>26</v>
       </c>
       <c r="G58" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H58" s="6" t="s">
         <v>21</v>
@@ -3843,7 +3843,7 @@
         <v>27</v>
       </c>
       <c r="G59" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H59" s="6" t="s">
         <v>21</v>
@@ -3884,7 +3884,7 @@
         <v>28</v>
       </c>
       <c r="G60" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H60" s="6" t="s">
         <v>21</v>
@@ -3978,7 +3978,7 @@
         <v>26</v>
       </c>
       <c r="G62" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H62" s="6" t="s">
         <v>21</v>
@@ -4019,7 +4019,7 @@
         <v>27</v>
       </c>
       <c r="G63" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H63" s="6" t="s">
         <v>21</v>
@@ -4060,7 +4060,7 @@
         <v>28</v>
       </c>
       <c r="G64" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H64" s="6" t="s">
         <v>21</v>
@@ -4154,7 +4154,7 @@
         <v>26</v>
       </c>
       <c r="G66" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H66" s="6" t="s">
         <v>21</v>
@@ -4195,7 +4195,7 @@
         <v>27</v>
       </c>
       <c r="G67" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>21</v>
@@ -4236,7 +4236,7 @@
         <v>28</v>
       </c>
       <c r="G68" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H68" s="6" t="s">
         <v>21</v>
@@ -4330,7 +4330,7 @@
         <v>26</v>
       </c>
       <c r="G70" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>21</v>
@@ -4371,7 +4371,7 @@
         <v>27</v>
       </c>
       <c r="G71" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H71" s="6" t="s">
         <v>21</v>
@@ -4412,7 +4412,7 @@
         <v>28</v>
       </c>
       <c r="G72" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H72" s="6" t="s">
         <v>21</v>
@@ -4506,7 +4506,7 @@
         <v>26</v>
       </c>
       <c r="G74" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H74" s="6" t="s">
         <v>21</v>
@@ -4547,7 +4547,7 @@
         <v>27</v>
       </c>
       <c r="G75" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H75" s="6" t="s">
         <v>21</v>
@@ -4588,7 +4588,7 @@
         <v>28</v>
       </c>
       <c r="G76" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H76" s="6" t="s">
         <v>21</v>
@@ -4682,7 +4682,7 @@
         <v>26</v>
       </c>
       <c r="G78" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H78" s="6" t="s">
         <v>21</v>
@@ -4723,7 +4723,7 @@
         <v>27</v>
       </c>
       <c r="G79" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H79" s="6" t="s">
         <v>21</v>
@@ -4764,7 +4764,7 @@
         <v>28</v>
       </c>
       <c r="G80" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H80" s="6" t="s">
         <v>21</v>
@@ -4858,7 +4858,7 @@
         <v>26</v>
       </c>
       <c r="G82" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H82" s="6" t="s">
         <v>21</v>
@@ -4899,7 +4899,7 @@
         <v>27</v>
       </c>
       <c r="G83" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H83" s="6" t="s">
         <v>21</v>
@@ -4940,7 +4940,7 @@
         <v>28</v>
       </c>
       <c r="G84" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H84" s="6" t="s">
         <v>21</v>
@@ -5087,7 +5087,7 @@
         <v>26</v>
       </c>
       <c r="G87" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H87" s="6" t="s">
         <v>21</v>
@@ -5128,7 +5128,7 @@
         <v>27</v>
       </c>
       <c r="G88" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H88" s="6" t="s">
         <v>21</v>
@@ -5169,7 +5169,7 @@
         <v>28</v>
       </c>
       <c r="G89" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H89" s="6" t="s">
         <v>21</v>
@@ -5263,7 +5263,7 @@
         <v>26</v>
       </c>
       <c r="G91" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H91" s="6" t="s">
         <v>21</v>
@@ -5304,7 +5304,7 @@
         <v>27</v>
       </c>
       <c r="G92" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H92" s="6" t="s">
         <v>21</v>
@@ -5345,7 +5345,7 @@
         <v>28</v>
       </c>
       <c r="G93" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H93" s="6" t="s">
         <v>21</v>
@@ -5439,7 +5439,7 @@
         <v>26</v>
       </c>
       <c r="G95" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H95" s="6" t="s">
         <v>21</v>
@@ -5480,7 +5480,7 @@
         <v>27</v>
       </c>
       <c r="G96" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H96" s="6" t="s">
         <v>21</v>
@@ -5521,7 +5521,7 @@
         <v>28</v>
       </c>
       <c r="G97" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H97" s="6" t="s">
         <v>21</v>
@@ -5615,7 +5615,7 @@
         <v>26</v>
       </c>
       <c r="G99" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H99" s="6" t="s">
         <v>21</v>
@@ -5656,7 +5656,7 @@
         <v>27</v>
       </c>
       <c r="G100" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H100" s="6" t="s">
         <v>21</v>
@@ -5697,7 +5697,7 @@
         <v>28</v>
       </c>
       <c r="G101" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H101" s="6" t="s">
         <v>21</v>
@@ -5791,7 +5791,7 @@
         <v>26</v>
       </c>
       <c r="G103" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H103" s="6" t="s">
         <v>21</v>
@@ -5832,7 +5832,7 @@
         <v>27</v>
       </c>
       <c r="G104" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H104" s="6" t="s">
         <v>21</v>
@@ -5873,7 +5873,7 @@
         <v>28</v>
       </c>
       <c r="G105" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H105" s="6" t="s">
         <v>21</v>
@@ -5967,7 +5967,7 @@
         <v>26</v>
       </c>
       <c r="G107" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H107" s="6" t="s">
         <v>21</v>
@@ -6008,7 +6008,7 @@
         <v>27</v>
       </c>
       <c r="G108" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H108" s="6" t="s">
         <v>21</v>
@@ -6049,7 +6049,7 @@
         <v>28</v>
       </c>
       <c r="G109" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H109" s="6" t="s">
         <v>21</v>
@@ -6143,7 +6143,7 @@
         <v>26</v>
       </c>
       <c r="G111" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H111" s="6" t="s">
         <v>21</v>
@@ -6184,7 +6184,7 @@
         <v>27</v>
       </c>
       <c r="G112" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H112" s="6" t="s">
         <v>21</v>
@@ -6225,7 +6225,7 @@
         <v>28</v>
       </c>
       <c r="G113" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H113" s="6" t="s">
         <v>21</v>
@@ -6319,7 +6319,7 @@
         <v>26</v>
       </c>
       <c r="G115" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H115" s="6" t="s">
         <v>21</v>
@@ -6360,7 +6360,7 @@
         <v>27</v>
       </c>
       <c r="G116" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H116" s="6" t="s">
         <v>21</v>
@@ -6401,7 +6401,7 @@
         <v>28</v>
       </c>
       <c r="G117" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H117" s="6" t="s">
         <v>21</v>
@@ -6495,7 +6495,7 @@
         <v>26</v>
       </c>
       <c r="G119" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H119" s="6" t="s">
         <v>21</v>
@@ -6536,7 +6536,7 @@
         <v>27</v>
       </c>
       <c r="G120" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H120" s="6" t="s">
         <v>21</v>
@@ -6577,7 +6577,7 @@
         <v>28</v>
       </c>
       <c r="G121" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H121" s="6" t="s">
         <v>21</v>
@@ -6671,7 +6671,7 @@
         <v>26</v>
       </c>
       <c r="G123" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H123" s="6" t="s">
         <v>21</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="G124" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H124" s="6" t="s">
         <v>21</v>
@@ -6753,7 +6753,7 @@
         <v>28</v>
       </c>
       <c r="G125" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H125" s="6" t="s">
         <v>21</v>
@@ -6900,7 +6900,7 @@
         <v>26</v>
       </c>
       <c r="G128" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H128" s="6" t="s">
         <v>21</v>
@@ -6941,7 +6941,7 @@
         <v>27</v>
       </c>
       <c r="G129" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H129" s="6" t="s">
         <v>21</v>
@@ -6982,7 +6982,7 @@
         <v>28</v>
       </c>
       <c r="G130" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H130" s="6" t="s">
         <v>21</v>
@@ -7076,7 +7076,7 @@
         <v>26</v>
       </c>
       <c r="G132" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H132" s="6" t="s">
         <v>21</v>
@@ -7117,7 +7117,7 @@
         <v>27</v>
       </c>
       <c r="G133" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H133" s="6" t="s">
         <v>21</v>
@@ -7158,7 +7158,7 @@
         <v>28</v>
       </c>
       <c r="G134" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H134" s="6" t="s">
         <v>21</v>
@@ -7252,7 +7252,7 @@
         <v>26</v>
       </c>
       <c r="G136" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H136" s="6" t="s">
         <v>21</v>
@@ -7293,7 +7293,7 @@
         <v>27</v>
       </c>
       <c r="G137" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H137" s="6" t="s">
         <v>21</v>
@@ -7334,7 +7334,7 @@
         <v>28</v>
       </c>
       <c r="G138" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H138" s="6" t="s">
         <v>21</v>
@@ -7428,7 +7428,7 @@
         <v>26</v>
       </c>
       <c r="G140" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H140" s="6" t="s">
         <v>21</v>
@@ -7469,7 +7469,7 @@
         <v>27</v>
       </c>
       <c r="G141" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H141" s="6" t="s">
         <v>21</v>
@@ -7510,7 +7510,7 @@
         <v>28</v>
       </c>
       <c r="G142" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H142" s="6" t="s">
         <v>21</v>
@@ -7556,8 +7556,10 @@
       <c r="C143" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D143" s="6" t="s">
-        <v>80</v>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>Молот великанов</t>
+        </is>
       </c>
       <c r="E143" s="6">
         <v>25</v>
@@ -7604,7 +7606,7 @@
         <v>26</v>
       </c>
       <c r="G144" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H144" s="6" t="s">
         <v>21</v>
@@ -7645,7 +7647,7 @@
         <v>27</v>
       </c>
       <c r="G145" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H145" s="6" t="s">
         <v>21</v>
@@ -7686,7 +7688,7 @@
         <v>28</v>
       </c>
       <c r="G146" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H146" s="6" t="s">
         <v>21</v>
@@ -7780,7 +7782,7 @@
         <v>26</v>
       </c>
       <c r="G148" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H148" s="6" t="s">
         <v>21</v>
@@ -7821,7 +7823,7 @@
         <v>27</v>
       </c>
       <c r="G149" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H149" s="6" t="s">
         <v>21</v>
@@ -7862,7 +7864,7 @@
         <v>28</v>
       </c>
       <c r="G150" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H150" s="6" t="s">
         <v>21</v>
@@ -7956,7 +7958,7 @@
         <v>26</v>
       </c>
       <c r="G152" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H152" s="6" t="s">
         <v>21</v>
@@ -7997,7 +7999,7 @@
         <v>27</v>
       </c>
       <c r="G153" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H153" s="6" t="s">
         <v>21</v>
@@ -8038,7 +8040,7 @@
         <v>28</v>
       </c>
       <c r="G154" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H154" s="6" t="s">
         <v>21</v>
@@ -8132,7 +8134,7 @@
         <v>26</v>
       </c>
       <c r="G156" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H156" s="6" t="s">
         <v>21</v>
@@ -8173,7 +8175,7 @@
         <v>27</v>
       </c>
       <c r="G157" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H157" s="6" t="s">
         <v>21</v>
@@ -8214,7 +8216,7 @@
         <v>28</v>
       </c>
       <c r="G158" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H158" s="6" t="s">
         <v>21</v>
@@ -8260,8 +8262,10 @@
       <c r="C159" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D159" s="6" t="s">
-        <v>84</v>
+      <c r="D159" s="6" t="inlineStr">
+        <is>
+          <t>Громовой молот</t>
+        </is>
       </c>
       <c r="E159" s="6">
         <v>45</v>
@@ -8308,7 +8312,7 @@
         <v>26</v>
       </c>
       <c r="G160" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H160" s="6" t="s">
         <v>21</v>
@@ -8349,7 +8353,7 @@
         <v>27</v>
       </c>
       <c r="G161" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H161" s="6" t="s">
         <v>21</v>
@@ -8390,7 +8394,7 @@
         <v>28</v>
       </c>
       <c r="G162" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H162" s="6" t="s">
         <v>21</v>
@@ -8484,7 +8488,7 @@
         <v>26</v>
       </c>
       <c r="G164" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H164" s="6" t="s">
         <v>21</v>
@@ -8525,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="G165" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H165" s="6" t="s">
         <v>21</v>
@@ -8566,7 +8570,7 @@
         <v>28</v>
       </c>
       <c r="G166" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H166" s="6" t="s">
         <v>21</v>
@@ -8713,7 +8717,7 @@
         <v>26</v>
       </c>
       <c r="G169" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H169" s="6" t="s">
         <v>21</v>
@@ -8754,7 +8758,7 @@
         <v>27</v>
       </c>
       <c r="G170" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H170" s="6" t="s">
         <v>21</v>
@@ -8795,7 +8799,7 @@
         <v>28</v>
       </c>
       <c r="G171" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H171" s="6" t="s">
         <v>21</v>
@@ -8889,7 +8893,7 @@
         <v>26</v>
       </c>
       <c r="G173" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H173" s="6" t="s">
         <v>21</v>
@@ -8930,7 +8934,7 @@
         <v>27</v>
       </c>
       <c r="G174" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H174" s="6" t="s">
         <v>21</v>
@@ -8971,7 +8975,7 @@
         <v>28</v>
       </c>
       <c r="G175" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H175" s="6" t="s">
         <v>21</v>
@@ -9065,7 +9069,7 @@
         <v>26</v>
       </c>
       <c r="G177" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H177" s="6" t="s">
         <v>21</v>
@@ -9106,7 +9110,7 @@
         <v>27</v>
       </c>
       <c r="G178" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H178" s="6" t="s">
         <v>21</v>
@@ -9147,7 +9151,7 @@
         <v>28</v>
       </c>
       <c r="G179" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H179" s="6" t="s">
         <v>21</v>
@@ -9241,7 +9245,7 @@
         <v>26</v>
       </c>
       <c r="G181" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H181" s="6" t="s">
         <v>21</v>
@@ -9282,7 +9286,7 @@
         <v>27</v>
       </c>
       <c r="G182" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H182" s="6" t="s">
         <v>21</v>
@@ -9323,7 +9327,7 @@
         <v>28</v>
       </c>
       <c r="G183" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H183" s="6" t="s">
         <v>21</v>
@@ -9417,7 +9421,7 @@
         <v>26</v>
       </c>
       <c r="G185" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H185" s="6" t="s">
         <v>21</v>
@@ -9458,7 +9462,7 @@
         <v>27</v>
       </c>
       <c r="G186" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H186" s="6" t="s">
         <v>21</v>
@@ -9499,7 +9503,7 @@
         <v>28</v>
       </c>
       <c r="G187" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H187" s="6" t="s">
         <v>21</v>
@@ -9593,7 +9597,7 @@
         <v>26</v>
       </c>
       <c r="G189" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H189" s="6" t="s">
         <v>21</v>
@@ -9634,7 +9638,7 @@
         <v>27</v>
       </c>
       <c r="G190" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H190" s="6" t="s">
         <v>21</v>
@@ -9675,7 +9679,7 @@
         <v>28</v>
       </c>
       <c r="G191" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H191" s="6" t="s">
         <v>21</v>
@@ -9769,7 +9773,7 @@
         <v>26</v>
       </c>
       <c r="G193" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H193" s="6" t="s">
         <v>21</v>
@@ -9810,7 +9814,7 @@
         <v>27</v>
       </c>
       <c r="G194" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H194" s="6" t="s">
         <v>21</v>
@@ -9851,7 +9855,7 @@
         <v>28</v>
       </c>
       <c r="G195" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H195" s="6" t="s">
         <v>21</v>
@@ -9945,7 +9949,7 @@
         <v>26</v>
       </c>
       <c r="G197" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H197" s="6" t="s">
         <v>21</v>
@@ -9986,7 +9990,7 @@
         <v>27</v>
       </c>
       <c r="G198" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H198" s="6" t="s">
         <v>21</v>
@@ -10027,7 +10031,7 @@
         <v>28</v>
       </c>
       <c r="G199" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H199" s="6" t="s">
         <v>21</v>
@@ -10121,7 +10125,7 @@
         <v>26</v>
       </c>
       <c r="G201" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H201" s="6" t="s">
         <v>21</v>
@@ -10162,7 +10166,7 @@
         <v>27</v>
       </c>
       <c r="G202" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H202" s="6" t="s">
         <v>21</v>
@@ -10203,7 +10207,7 @@
         <v>28</v>
       </c>
       <c r="G203" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H203" s="6" t="s">
         <v>21</v>
@@ -10297,7 +10301,7 @@
         <v>26</v>
       </c>
       <c r="G205" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H205" s="6" t="s">
         <v>21</v>
@@ -10338,7 +10342,7 @@
         <v>27</v>
       </c>
       <c r="G206" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H206" s="6" t="s">
         <v>21</v>
@@ -10379,7 +10383,7 @@
         <v>28</v>
       </c>
       <c r="G207" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H207" s="6" t="s">
         <v>21</v>
@@ -10529,7 +10533,7 @@
         <v>21</v>
       </c>
       <c r="H210" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="I210" s="6" t="s">
         <v>21</v>
@@ -10570,7 +10574,7 @@
         <v>21</v>
       </c>
       <c r="H211" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="I211" s="6" t="s">
         <v>21</v>
@@ -10611,7 +10615,7 @@
         <v>21</v>
       </c>
       <c r="H212" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="I212" s="6" t="s">
         <v>21</v>
@@ -10705,7 +10709,7 @@
         <v>21</v>
       </c>
       <c r="H214" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="I214" s="6" t="s">
         <v>21</v>
@@ -10746,7 +10750,7 @@
         <v>21</v>
       </c>
       <c r="H215" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="I215" s="6" t="s">
         <v>21</v>
@@ -10787,7 +10791,7 @@
         <v>21</v>
       </c>
       <c r="H216" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="I216" s="6" t="s">
         <v>21</v>
@@ -10881,7 +10885,7 @@
         <v>21</v>
       </c>
       <c r="H218" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="I218" s="6" t="s">
         <v>21</v>
@@ -10922,7 +10926,7 @@
         <v>21</v>
       </c>
       <c r="H219" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="I219" s="6" t="s">
         <v>21</v>
@@ -10963,7 +10967,7 @@
         <v>21</v>
       </c>
       <c r="H220" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="I220" s="6" t="s">
         <v>21</v>
@@ -11057,7 +11061,7 @@
         <v>21</v>
       </c>
       <c r="H222" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="I222" s="6" t="s">
         <v>21</v>
@@ -11098,7 +11102,7 @@
         <v>21</v>
       </c>
       <c r="H223" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="I223" s="6" t="s">
         <v>21</v>
@@ -11139,7 +11143,7 @@
         <v>21</v>
       </c>
       <c r="H224" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="I224" s="6" t="s">
         <v>21</v>
@@ -11233,7 +11237,7 @@
         <v>21</v>
       </c>
       <c r="H226" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="I226" s="6" t="s">
         <v>21</v>
@@ -11274,7 +11278,7 @@
         <v>21</v>
       </c>
       <c r="H227" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="I227" s="6" t="s">
         <v>21</v>
@@ -11315,7 +11319,7 @@
         <v>21</v>
       </c>
       <c r="H228" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="I228" s="6" t="s">
         <v>21</v>
@@ -11409,7 +11413,7 @@
         <v>21</v>
       </c>
       <c r="H230" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="I230" s="6" t="s">
         <v>21</v>
@@ -11450,7 +11454,7 @@
         <v>21</v>
       </c>
       <c r="H231" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="I231" s="6" t="s">
         <v>21</v>
@@ -11491,7 +11495,7 @@
         <v>21</v>
       </c>
       <c r="H232" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="I232" s="6" t="s">
         <v>21</v>
@@ -11585,7 +11589,7 @@
         <v>21</v>
       </c>
       <c r="H234" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="I234" s="6" t="s">
         <v>21</v>
@@ -11626,7 +11630,7 @@
         <v>21</v>
       </c>
       <c r="H235" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="I235" s="6" t="s">
         <v>21</v>
@@ -11667,7 +11671,7 @@
         <v>21</v>
       </c>
       <c r="H236" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="I236" s="6" t="s">
         <v>21</v>
@@ -11761,7 +11765,7 @@
         <v>21</v>
       </c>
       <c r="H238" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="I238" s="6" t="s">
         <v>21</v>
@@ -11802,7 +11806,7 @@
         <v>21</v>
       </c>
       <c r="H239" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="I239" s="6" t="s">
         <v>21</v>
@@ -11843,7 +11847,7 @@
         <v>21</v>
       </c>
       <c r="H240" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="I240" s="6" t="s">
         <v>21</v>
@@ -11937,7 +11941,7 @@
         <v>21</v>
       </c>
       <c r="H242" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="I242" s="6" t="s">
         <v>21</v>
@@ -11978,7 +11982,7 @@
         <v>21</v>
       </c>
       <c r="H243" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="I243" s="6" t="s">
         <v>21</v>
@@ -12019,7 +12023,7 @@
         <v>21</v>
       </c>
       <c r="H244" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="I244" s="6" t="s">
         <v>21</v>
@@ -12113,7 +12117,7 @@
         <v>21</v>
       </c>
       <c r="H246" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="I246" s="6" t="s">
         <v>21</v>
@@ -12154,7 +12158,7 @@
         <v>21</v>
       </c>
       <c r="H247" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="I247" s="6" t="s">
         <v>21</v>
@@ -12195,7 +12199,7 @@
         <v>21</v>
       </c>
       <c r="H248" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="I248" s="6" t="s">
         <v>21</v>
@@ -12348,7 +12352,7 @@
         <v>21</v>
       </c>
       <c r="J251" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="K251" s="6">
         <v>1</v>
@@ -12389,7 +12393,7 @@
         <v>21</v>
       </c>
       <c r="J252" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="K252" s="6">
         <v>1</v>
@@ -12430,7 +12434,7 @@
         <v>21</v>
       </c>
       <c r="J253" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="K253" s="6">
         <v>1</v>
@@ -12524,7 +12528,7 @@
         <v>21</v>
       </c>
       <c r="J255" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="K255" s="6">
         <v>1</v>
@@ -12565,7 +12569,7 @@
         <v>21</v>
       </c>
       <c r="J256" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="K256" s="6">
         <v>1</v>
@@ -12606,7 +12610,7 @@
         <v>21</v>
       </c>
       <c r="J257" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="K257" s="6">
         <v>1</v>
@@ -12700,7 +12704,7 @@
         <v>21</v>
       </c>
       <c r="J259" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="K259" s="6">
         <v>1</v>
@@ -12741,7 +12745,7 @@
         <v>21</v>
       </c>
       <c r="J260" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="K260" s="6">
         <v>1</v>
@@ -12782,7 +12786,7 @@
         <v>21</v>
       </c>
       <c r="J261" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="K261" s="6">
         <v>1</v>
@@ -12876,7 +12880,7 @@
         <v>21</v>
       </c>
       <c r="J263" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="K263" s="6">
         <v>1</v>
@@ -12917,7 +12921,7 @@
         <v>21</v>
       </c>
       <c r="J264" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="K264" s="6">
         <v>1</v>
@@ -12958,7 +12962,7 @@
         <v>21</v>
       </c>
       <c r="J265" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="K265" s="6">
         <v>1</v>
@@ -13052,7 +13056,7 @@
         <v>21</v>
       </c>
       <c r="J267" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="K267" s="6">
         <v>1</v>
@@ -13093,7 +13097,7 @@
         <v>21</v>
       </c>
       <c r="J268" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="K268" s="6">
         <v>1</v>
@@ -13134,7 +13138,7 @@
         <v>21</v>
       </c>
       <c r="J269" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="K269" s="6">
         <v>1</v>
@@ -13228,7 +13232,7 @@
         <v>21</v>
       </c>
       <c r="J271" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="K271" s="6">
         <v>1</v>
@@ -13269,7 +13273,7 @@
         <v>21</v>
       </c>
       <c r="J272" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="K272" s="6">
         <v>1</v>
@@ -13310,7 +13314,7 @@
         <v>21</v>
       </c>
       <c r="J273" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="K273" s="6">
         <v>1</v>
@@ -13404,7 +13408,7 @@
         <v>21</v>
       </c>
       <c r="J275" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="K275" s="6">
         <v>1</v>
@@ -13445,7 +13449,7 @@
         <v>21</v>
       </c>
       <c r="J276" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="K276" s="6">
         <v>1</v>
@@ -13486,7 +13490,7 @@
         <v>21</v>
       </c>
       <c r="J277" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="K277" s="6">
         <v>1</v>
@@ -13580,7 +13584,7 @@
         <v>21</v>
       </c>
       <c r="J279" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="K279" s="6">
         <v>1</v>
@@ -13621,7 +13625,7 @@
         <v>21</v>
       </c>
       <c r="J280" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="K280" s="6">
         <v>1</v>
@@ -13662,7 +13666,7 @@
         <v>21</v>
       </c>
       <c r="J281" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="K281" s="6">
         <v>1</v>
@@ -13756,7 +13760,7 @@
         <v>21</v>
       </c>
       <c r="J283" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="K283" s="6">
         <v>1</v>
@@ -13797,7 +13801,7 @@
         <v>21</v>
       </c>
       <c r="J284" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="K284" s="6">
         <v>1</v>
@@ -13838,7 +13842,7 @@
         <v>21</v>
       </c>
       <c r="J285" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="K285" s="6">
         <v>1</v>
@@ -13932,7 +13936,7 @@
         <v>21</v>
       </c>
       <c r="J287" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="K287" s="6">
         <v>1</v>
@@ -13973,7 +13977,7 @@
         <v>21</v>
       </c>
       <c r="J288" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="K288" s="6">
         <v>1</v>
@@ -14014,7 +14018,7 @@
         <v>21</v>
       </c>
       <c r="J289" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="K289" s="6">
         <v>1</v>
@@ -14152,7 +14156,7 @@
         <v>26</v>
       </c>
       <c r="G292" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H292" s="6" t="s">
         <v>21</v>
@@ -14193,7 +14197,7 @@
         <v>27</v>
       </c>
       <c r="G293" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H293" s="6" t="s">
         <v>21</v>
@@ -14234,7 +14238,7 @@
         <v>28</v>
       </c>
       <c r="G294" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H294" s="6" t="s">
         <v>21</v>
@@ -14328,7 +14332,7 @@
         <v>26</v>
       </c>
       <c r="G296" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H296" s="6" t="s">
         <v>21</v>
@@ -14369,7 +14373,7 @@
         <v>27</v>
       </c>
       <c r="G297" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H297" s="6" t="s">
         <v>21</v>
@@ -14410,7 +14414,7 @@
         <v>28</v>
       </c>
       <c r="G298" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H298" s="6" t="s">
         <v>21</v>
@@ -14504,7 +14508,7 @@
         <v>26</v>
       </c>
       <c r="G300" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H300" s="6" t="s">
         <v>21</v>
@@ -14545,7 +14549,7 @@
         <v>27</v>
       </c>
       <c r="G301" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H301" s="6" t="s">
         <v>21</v>
@@ -14586,7 +14590,7 @@
         <v>28</v>
       </c>
       <c r="G302" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H302" s="6" t="s">
         <v>21</v>
@@ -14680,7 +14684,7 @@
         <v>26</v>
       </c>
       <c r="G304" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H304" s="6" t="s">
         <v>21</v>
@@ -14721,7 +14725,7 @@
         <v>27</v>
       </c>
       <c r="G305" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H305" s="6" t="s">
         <v>21</v>
@@ -14762,7 +14766,7 @@
         <v>28</v>
       </c>
       <c r="G306" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H306" s="6" t="s">
         <v>21</v>
@@ -14856,7 +14860,7 @@
         <v>26</v>
       </c>
       <c r="G308" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H308" s="6" t="s">
         <v>21</v>
@@ -14897,7 +14901,7 @@
         <v>27</v>
       </c>
       <c r="G309" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H309" s="6" t="s">
         <v>21</v>
@@ -14938,7 +14942,7 @@
         <v>28</v>
       </c>
       <c r="G310" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H310" s="6" t="s">
         <v>21</v>
@@ -15032,7 +15036,7 @@
         <v>26</v>
       </c>
       <c r="G312" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H312" s="6" t="s">
         <v>21</v>
@@ -15073,7 +15077,7 @@
         <v>27</v>
       </c>
       <c r="G313" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H313" s="6" t="s">
         <v>21</v>
@@ -15114,7 +15118,7 @@
         <v>28</v>
       </c>
       <c r="G314" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H314" s="6" t="s">
         <v>21</v>
@@ -15208,7 +15212,7 @@
         <v>26</v>
       </c>
       <c r="G316" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H316" s="6" t="s">
         <v>21</v>
@@ -15249,7 +15253,7 @@
         <v>27</v>
       </c>
       <c r="G317" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H317" s="6" t="s">
         <v>21</v>
@@ -15290,7 +15294,7 @@
         <v>28</v>
       </c>
       <c r="G318" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H318" s="6" t="s">
         <v>21</v>
@@ -15384,7 +15388,7 @@
         <v>26</v>
       </c>
       <c r="G320" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H320" s="6" t="s">
         <v>21</v>
@@ -15425,7 +15429,7 @@
         <v>27</v>
       </c>
       <c r="G321" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H321" s="6" t="s">
         <v>21</v>
@@ -15466,7 +15470,7 @@
         <v>28</v>
       </c>
       <c r="G322" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H322" s="6" t="s">
         <v>21</v>
@@ -15560,7 +15564,7 @@
         <v>26</v>
       </c>
       <c r="G324" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H324" s="6" t="s">
         <v>21</v>
@@ -15601,7 +15605,7 @@
         <v>27</v>
       </c>
       <c r="G325" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H325" s="6" t="s">
         <v>21</v>
@@ -15642,7 +15646,7 @@
         <v>28</v>
       </c>
       <c r="G326" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H326" s="6" t="s">
         <v>21</v>
@@ -15736,7 +15740,7 @@
         <v>26</v>
       </c>
       <c r="G328" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H328" s="6" t="s">
         <v>21</v>
@@ -15777,7 +15781,7 @@
         <v>27</v>
       </c>
       <c r="G329" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H329" s="6" t="s">
         <v>21</v>
@@ -15818,7 +15822,7 @@
         <v>28</v>
       </c>
       <c r="G330" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H330" s="6" t="s">
         <v>21</v>
@@ -15968,7 +15972,7 @@
         <v>21</v>
       </c>
       <c r="H333" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="I333" s="6" t="s">
         <v>21</v>
@@ -16009,7 +16013,7 @@
         <v>21</v>
       </c>
       <c r="H334" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="I334" s="6" t="s">
         <v>21</v>
@@ -16050,7 +16054,7 @@
         <v>21</v>
       </c>
       <c r="H335" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="I335" s="6" t="s">
         <v>21</v>
@@ -16144,7 +16148,7 @@
         <v>21</v>
       </c>
       <c r="H337" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="I337" s="6" t="s">
         <v>21</v>
@@ -16185,7 +16189,7 @@
         <v>21</v>
       </c>
       <c r="H338" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="I338" s="6" t="s">
         <v>21</v>
@@ -16226,7 +16230,7 @@
         <v>21</v>
       </c>
       <c r="H339" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="I339" s="6" t="s">
         <v>21</v>
@@ -16320,7 +16324,7 @@
         <v>21</v>
       </c>
       <c r="H341" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="I341" s="6" t="s">
         <v>21</v>
@@ -16361,7 +16365,7 @@
         <v>21</v>
       </c>
       <c r="H342" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="I342" s="6" t="s">
         <v>21</v>
@@ -16402,7 +16406,7 @@
         <v>21</v>
       </c>
       <c r="H343" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="I343" s="6" t="s">
         <v>21</v>
@@ -16496,7 +16500,7 @@
         <v>21</v>
       </c>
       <c r="H345" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="I345" s="6" t="s">
         <v>21</v>
@@ -16537,7 +16541,7 @@
         <v>21</v>
       </c>
       <c r="H346" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="I346" s="6" t="s">
         <v>21</v>
@@ -16578,7 +16582,7 @@
         <v>21</v>
       </c>
       <c r="H347" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="I347" s="6" t="s">
         <v>21</v>
@@ -16672,7 +16676,7 @@
         <v>21</v>
       </c>
       <c r="H349" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="I349" s="6" t="s">
         <v>21</v>
@@ -16713,7 +16717,7 @@
         <v>21</v>
       </c>
       <c r="H350" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="I350" s="6" t="s">
         <v>21</v>
@@ -16754,7 +16758,7 @@
         <v>21</v>
       </c>
       <c r="H351" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="I351" s="6" t="s">
         <v>21</v>
@@ -16848,7 +16852,7 @@
         <v>21</v>
       </c>
       <c r="H353" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="I353" s="6" t="s">
         <v>21</v>
@@ -16889,7 +16893,7 @@
         <v>21</v>
       </c>
       <c r="H354" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="I354" s="6" t="s">
         <v>21</v>
@@ -16930,7 +16934,7 @@
         <v>21</v>
       </c>
       <c r="H355" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="I355" s="6" t="s">
         <v>21</v>
@@ -17024,7 +17028,7 @@
         <v>21</v>
       </c>
       <c r="H357" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="I357" s="6" t="s">
         <v>21</v>
@@ -17065,7 +17069,7 @@
         <v>21</v>
       </c>
       <c r="H358" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="I358" s="6" t="s">
         <v>21</v>
@@ -17106,7 +17110,7 @@
         <v>21</v>
       </c>
       <c r="H359" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="I359" s="6" t="s">
         <v>21</v>
@@ -17200,7 +17204,7 @@
         <v>21</v>
       </c>
       <c r="H361" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="I361" s="6" t="s">
         <v>21</v>
@@ -17241,7 +17245,7 @@
         <v>21</v>
       </c>
       <c r="H362" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="I362" s="6" t="s">
         <v>21</v>
@@ -17282,7 +17286,7 @@
         <v>21</v>
       </c>
       <c r="H363" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="I363" s="6" t="s">
         <v>21</v>
@@ -17376,7 +17380,7 @@
         <v>21</v>
       </c>
       <c r="H365" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="I365" s="6" t="s">
         <v>21</v>
@@ -17417,7 +17421,7 @@
         <v>21</v>
       </c>
       <c r="H366" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="I366" s="6" t="s">
         <v>21</v>
@@ -17458,7 +17462,7 @@
         <v>21</v>
       </c>
       <c r="H367" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="I367" s="6" t="s">
         <v>21</v>
@@ -17552,7 +17556,7 @@
         <v>21</v>
       </c>
       <c r="H369" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="I369" s="6" t="s">
         <v>21</v>
@@ -17593,7 +17597,7 @@
         <v>21</v>
       </c>
       <c r="H370" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="I370" s="6" t="s">
         <v>21</v>
@@ -17634,7 +17638,7 @@
         <v>21</v>
       </c>
       <c r="H371" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="I371" s="6" t="s">
         <v>21</v>
@@ -17778,7 +17782,7 @@
         <v>26</v>
       </c>
       <c r="G374" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H374" s="6" t="s">
         <v>21</v>
@@ -17819,7 +17823,7 @@
         <v>27</v>
       </c>
       <c r="G375" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H375" s="6" t="s">
         <v>21</v>
@@ -17860,7 +17864,7 @@
         <v>28</v>
       </c>
       <c r="G376" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H376" s="6" t="s">
         <v>21</v>
@@ -17954,7 +17958,7 @@
         <v>26</v>
       </c>
       <c r="G378" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H378" s="6" t="s">
         <v>21</v>
@@ -17995,7 +17999,7 @@
         <v>27</v>
       </c>
       <c r="G379" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H379" s="6" t="s">
         <v>21</v>
@@ -18036,7 +18040,7 @@
         <v>28</v>
       </c>
       <c r="G380" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H380" s="6" t="s">
         <v>21</v>
@@ -18130,7 +18134,7 @@
         <v>26</v>
       </c>
       <c r="G382" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H382" s="6" t="s">
         <v>21</v>
@@ -18171,7 +18175,7 @@
         <v>27</v>
       </c>
       <c r="G383" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H383" s="6" t="s">
         <v>21</v>
@@ -18212,7 +18216,7 @@
         <v>28</v>
       </c>
       <c r="G384" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H384" s="6" t="s">
         <v>21</v>
@@ -18306,7 +18310,7 @@
         <v>26</v>
       </c>
       <c r="G386" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H386" s="6" t="s">
         <v>21</v>
@@ -18347,7 +18351,7 @@
         <v>27</v>
       </c>
       <c r="G387" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H387" s="6" t="s">
         <v>21</v>
@@ -18388,7 +18392,7 @@
         <v>28</v>
       </c>
       <c r="G388" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H388" s="6" t="s">
         <v>21</v>
@@ -18482,7 +18486,7 @@
         <v>26</v>
       </c>
       <c r="G390" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H390" s="6" t="s">
         <v>21</v>
@@ -18523,7 +18527,7 @@
         <v>27</v>
       </c>
       <c r="G391" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H391" s="6" t="s">
         <v>21</v>
@@ -18564,7 +18568,7 @@
         <v>28</v>
       </c>
       <c r="G392" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H392" s="6" t="s">
         <v>21</v>
@@ -18658,7 +18662,7 @@
         <v>26</v>
       </c>
       <c r="G394" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H394" s="6" t="s">
         <v>21</v>
@@ -18699,7 +18703,7 @@
         <v>27</v>
       </c>
       <c r="G395" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H395" s="6" t="s">
         <v>21</v>
@@ -18740,7 +18744,7 @@
         <v>28</v>
       </c>
       <c r="G396" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H396" s="6" t="s">
         <v>21</v>
@@ -18834,7 +18838,7 @@
         <v>26</v>
       </c>
       <c r="G398" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H398" s="6" t="s">
         <v>21</v>
@@ -18875,7 +18879,7 @@
         <v>27</v>
       </c>
       <c r="G399" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H399" s="6" t="s">
         <v>21</v>
@@ -18916,7 +18920,7 @@
         <v>28</v>
       </c>
       <c r="G400" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H400" s="6" t="s">
         <v>21</v>
@@ -19010,7 +19014,7 @@
         <v>26</v>
       </c>
       <c r="G402" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H402" s="6" t="s">
         <v>21</v>
@@ -19051,7 +19055,7 @@
         <v>27</v>
       </c>
       <c r="G403" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H403" s="6" t="s">
         <v>21</v>
@@ -19092,7 +19096,7 @@
         <v>28</v>
       </c>
       <c r="G404" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H404" s="6" t="s">
         <v>21</v>
@@ -19186,7 +19190,7 @@
         <v>26</v>
       </c>
       <c r="G406" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H406" s="6" t="s">
         <v>21</v>
@@ -19227,7 +19231,7 @@
         <v>27</v>
       </c>
       <c r="G407" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H407" s="6" t="s">
         <v>21</v>
@@ -19268,7 +19272,7 @@
         <v>28</v>
       </c>
       <c r="G408" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H408" s="6" t="s">
         <v>21</v>
@@ -19362,7 +19366,7 @@
         <v>26</v>
       </c>
       <c r="G410" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H410" s="6" t="s">
         <v>21</v>
@@ -19403,7 +19407,7 @@
         <v>27</v>
       </c>
       <c r="G411" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H411" s="6" t="s">
         <v>21</v>
@@ -19444,7 +19448,7 @@
         <v>28</v>
       </c>
       <c r="G412" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H412" s="6" t="s">
         <v>21</v>
@@ -19591,7 +19595,7 @@
         <v>26</v>
       </c>
       <c r="G415" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H415" s="6" t="s">
         <v>21</v>
@@ -19632,7 +19636,7 @@
         <v>27</v>
       </c>
       <c r="G416" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H416" s="6" t="s">
         <v>21</v>
@@ -19673,7 +19677,7 @@
         <v>28</v>
       </c>
       <c r="G417" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H417" s="6" t="s">
         <v>21</v>
@@ -19767,7 +19771,7 @@
         <v>26</v>
       </c>
       <c r="G419" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H419" s="6" t="s">
         <v>21</v>
@@ -19808,7 +19812,7 @@
         <v>27</v>
       </c>
       <c r="G420" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H420" s="6" t="s">
         <v>21</v>
@@ -19849,7 +19853,7 @@
         <v>28</v>
       </c>
       <c r="G421" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H421" s="6" t="s">
         <v>21</v>
@@ -19943,7 +19947,7 @@
         <v>26</v>
       </c>
       <c r="G423" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H423" s="6" t="s">
         <v>21</v>
@@ -19984,7 +19988,7 @@
         <v>27</v>
       </c>
       <c r="G424" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H424" s="6" t="s">
         <v>21</v>
@@ -20025,7 +20029,7 @@
         <v>28</v>
       </c>
       <c r="G425" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H425" s="6" t="s">
         <v>21</v>
@@ -20119,7 +20123,7 @@
         <v>26</v>
       </c>
       <c r="G427" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H427" s="6" t="s">
         <v>21</v>
@@ -20160,7 +20164,7 @@
         <v>27</v>
       </c>
       <c r="G428" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H428" s="6" t="s">
         <v>21</v>
@@ -20201,7 +20205,7 @@
         <v>28</v>
       </c>
       <c r="G429" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H429" s="6" t="s">
         <v>21</v>
@@ -20295,7 +20299,7 @@
         <v>26</v>
       </c>
       <c r="G431" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H431" s="6" t="s">
         <v>21</v>
@@ -20336,7 +20340,7 @@
         <v>27</v>
       </c>
       <c r="G432" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H432" s="6" t="s">
         <v>21</v>
@@ -20377,7 +20381,7 @@
         <v>28</v>
       </c>
       <c r="G433" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H433" s="6" t="s">
         <v>21</v>
@@ -20471,7 +20475,7 @@
         <v>26</v>
       </c>
       <c r="G435" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H435" s="6" t="s">
         <v>21</v>
@@ -20512,7 +20516,7 @@
         <v>27</v>
       </c>
       <c r="G436" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H436" s="6" t="s">
         <v>21</v>
@@ -20553,7 +20557,7 @@
         <v>28</v>
       </c>
       <c r="G437" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H437" s="6" t="s">
         <v>21</v>
@@ -20647,7 +20651,7 @@
         <v>26</v>
       </c>
       <c r="G439" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H439" s="6" t="s">
         <v>21</v>
@@ -20688,7 +20692,7 @@
         <v>27</v>
       </c>
       <c r="G440" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H440" s="6" t="s">
         <v>21</v>
@@ -20729,7 +20733,7 @@
         <v>28</v>
       </c>
       <c r="G441" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H441" s="6" t="s">
         <v>21</v>
@@ -20823,7 +20827,7 @@
         <v>26</v>
       </c>
       <c r="G443" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H443" s="6" t="s">
         <v>21</v>
@@ -20864,7 +20868,7 @@
         <v>27</v>
       </c>
       <c r="G444" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H444" s="6" t="s">
         <v>21</v>
@@ -20905,7 +20909,7 @@
         <v>28</v>
       </c>
       <c r="G445" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H445" s="6" t="s">
         <v>21</v>
@@ -20999,7 +21003,7 @@
         <v>26</v>
       </c>
       <c r="G447" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H447" s="6" t="s">
         <v>21</v>
@@ -21040,7 +21044,7 @@
         <v>27</v>
       </c>
       <c r="G448" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H448" s="6" t="s">
         <v>21</v>
@@ -21081,7 +21085,7 @@
         <v>28</v>
       </c>
       <c r="G449" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H449" s="6" t="s">
         <v>21</v>
@@ -21175,7 +21179,7 @@
         <v>26</v>
       </c>
       <c r="G451" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H451" s="6" t="s">
         <v>21</v>
@@ -21216,7 +21220,7 @@
         <v>27</v>
       </c>
       <c r="G452" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H452" s="6" t="s">
         <v>21</v>
@@ -21257,7 +21261,7 @@
         <v>28</v>
       </c>
       <c r="G453" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H453" s="6" t="s">
         <v>21</v>
@@ -21404,7 +21408,7 @@
         <v>26</v>
       </c>
       <c r="G456" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H456" s="6" t="s">
         <v>21</v>
@@ -21445,7 +21449,7 @@
         <v>27</v>
       </c>
       <c r="G457" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H457" s="6" t="s">
         <v>21</v>
@@ -21486,7 +21490,7 @@
         <v>28</v>
       </c>
       <c r="G458" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H458" s="6" t="s">
         <v>21</v>
@@ -21580,7 +21584,7 @@
         <v>26</v>
       </c>
       <c r="G460" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H460" s="6" t="s">
         <v>21</v>
@@ -21621,7 +21625,7 @@
         <v>27</v>
       </c>
       <c r="G461" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H461" s="6" t="s">
         <v>21</v>
@@ -21662,7 +21666,7 @@
         <v>28</v>
       </c>
       <c r="G462" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H462" s="6" t="s">
         <v>21</v>
@@ -21756,7 +21760,7 @@
         <v>26</v>
       </c>
       <c r="G464" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H464" s="6" t="s">
         <v>21</v>
@@ -21797,7 +21801,7 @@
         <v>27</v>
       </c>
       <c r="G465" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H465" s="6" t="s">
         <v>21</v>
@@ -21838,7 +21842,7 @@
         <v>28</v>
       </c>
       <c r="G466" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H466" s="6" t="s">
         <v>21</v>
@@ -21932,7 +21936,7 @@
         <v>26</v>
       </c>
       <c r="G468" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H468" s="6" t="s">
         <v>21</v>
@@ -21973,7 +21977,7 @@
         <v>27</v>
       </c>
       <c r="G469" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H469" s="6" t="s">
         <v>21</v>
@@ -22014,7 +22018,7 @@
         <v>28</v>
       </c>
       <c r="G470" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H470" s="6" t="s">
         <v>21</v>
@@ -22108,7 +22112,7 @@
         <v>26</v>
       </c>
       <c r="G472" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H472" s="6" t="s">
         <v>21</v>
@@ -22149,7 +22153,7 @@
         <v>27</v>
       </c>
       <c r="G473" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H473" s="6" t="s">
         <v>21</v>
@@ -22190,7 +22194,7 @@
         <v>28</v>
       </c>
       <c r="G474" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H474" s="6" t="s">
         <v>21</v>
@@ -22284,7 +22288,7 @@
         <v>26</v>
       </c>
       <c r="G476" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H476" s="6" t="s">
         <v>21</v>
@@ -22325,7 +22329,7 @@
         <v>27</v>
       </c>
       <c r="G477" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H477" s="6" t="s">
         <v>21</v>
@@ -22366,7 +22370,7 @@
         <v>28</v>
       </c>
       <c r="G478" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H478" s="6" t="s">
         <v>21</v>
@@ -22460,7 +22464,7 @@
         <v>26</v>
       </c>
       <c r="G480" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H480" s="6" t="s">
         <v>21</v>
@@ -22501,7 +22505,7 @@
         <v>27</v>
       </c>
       <c r="G481" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H481" s="6" t="s">
         <v>21</v>
@@ -22542,7 +22546,7 @@
         <v>28</v>
       </c>
       <c r="G482" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H482" s="6" t="s">
         <v>21</v>
@@ -22636,7 +22640,7 @@
         <v>26</v>
       </c>
       <c r="G484" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H484" s="6" t="s">
         <v>21</v>
@@ -22677,7 +22681,7 @@
         <v>27</v>
       </c>
       <c r="G485" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H485" s="6" t="s">
         <v>21</v>
@@ -22718,7 +22722,7 @@
         <v>28</v>
       </c>
       <c r="G486" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H486" s="6" t="s">
         <v>21</v>
@@ -22812,7 +22816,7 @@
         <v>26</v>
       </c>
       <c r="G488" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H488" s="6" t="s">
         <v>21</v>
@@ -22853,7 +22857,7 @@
         <v>27</v>
       </c>
       <c r="G489" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H489" s="6" t="s">
         <v>21</v>
@@ -22894,7 +22898,7 @@
         <v>28</v>
       </c>
       <c r="G490" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H490" s="6" t="s">
         <v>21</v>
@@ -22988,7 +22992,7 @@
         <v>26</v>
       </c>
       <c r="G492" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H492" s="6" t="s">
         <v>21</v>
@@ -23029,7 +23033,7 @@
         <v>27</v>
       </c>
       <c r="G493" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H493" s="6" t="s">
         <v>21</v>
@@ -23070,7 +23074,7 @@
         <v>28</v>
       </c>
       <c r="G494" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H494" s="6" t="s">
         <v>21</v>
@@ -23217,7 +23221,7 @@
         <v>26</v>
       </c>
       <c r="G497" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H497" s="6" t="s">
         <v>21</v>
@@ -23258,7 +23262,7 @@
         <v>27</v>
       </c>
       <c r="G498" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H498" s="6" t="s">
         <v>21</v>
@@ -23299,7 +23303,7 @@
         <v>28</v>
       </c>
       <c r="G499" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H499" s="6" t="s">
         <v>21</v>
@@ -23393,7 +23397,7 @@
         <v>26</v>
       </c>
       <c r="G501" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H501" s="6" t="s">
         <v>21</v>
@@ -23434,7 +23438,7 @@
         <v>27</v>
       </c>
       <c r="G502" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H502" s="6" t="s">
         <v>21</v>
@@ -23475,7 +23479,7 @@
         <v>28</v>
       </c>
       <c r="G503" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H503" s="6" t="s">
         <v>21</v>
@@ -23569,7 +23573,7 @@
         <v>26</v>
       </c>
       <c r="G505" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H505" s="6" t="s">
         <v>21</v>
@@ -23610,7 +23614,7 @@
         <v>27</v>
       </c>
       <c r="G506" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H506" s="6" t="s">
         <v>21</v>
@@ -23651,7 +23655,7 @@
         <v>28</v>
       </c>
       <c r="G507" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H507" s="6" t="s">
         <v>21</v>
@@ -23745,7 +23749,7 @@
         <v>26</v>
       </c>
       <c r="G509" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H509" s="6" t="s">
         <v>21</v>
@@ -23786,7 +23790,7 @@
         <v>27</v>
       </c>
       <c r="G510" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H510" s="6" t="s">
         <v>21</v>
@@ -23827,7 +23831,7 @@
         <v>28</v>
       </c>
       <c r="G511" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H511" s="6" t="s">
         <v>21</v>
@@ -23921,7 +23925,7 @@
         <v>26</v>
       </c>
       <c r="G513" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H513" s="6" t="s">
         <v>21</v>
@@ -23962,7 +23966,7 @@
         <v>27</v>
       </c>
       <c r="G514" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H514" s="6" t="s">
         <v>21</v>
@@ -24003,7 +24007,7 @@
         <v>28</v>
       </c>
       <c r="G515" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H515" s="6" t="s">
         <v>21</v>
@@ -24097,7 +24101,7 @@
         <v>26</v>
       </c>
       <c r="G517" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H517" s="6" t="s">
         <v>21</v>
@@ -24138,7 +24142,7 @@
         <v>27</v>
       </c>
       <c r="G518" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H518" s="6" t="s">
         <v>21</v>
@@ -24179,7 +24183,7 @@
         <v>28</v>
       </c>
       <c r="G519" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H519" s="6" t="s">
         <v>21</v>
@@ -24273,7 +24277,7 @@
         <v>26</v>
       </c>
       <c r="G521" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H521" s="6" t="s">
         <v>21</v>
@@ -24314,7 +24318,7 @@
         <v>27</v>
       </c>
       <c r="G522" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H522" s="6" t="s">
         <v>21</v>
@@ -24355,7 +24359,7 @@
         <v>28</v>
       </c>
       <c r="G523" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H523" s="6" t="s">
         <v>21</v>
@@ -24449,7 +24453,7 @@
         <v>26</v>
       </c>
       <c r="G525" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H525" s="6" t="s">
         <v>21</v>
@@ -24490,7 +24494,7 @@
         <v>27</v>
       </c>
       <c r="G526" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H526" s="6" t="s">
         <v>21</v>
@@ -24531,7 +24535,7 @@
         <v>28</v>
       </c>
       <c r="G527" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H527" s="6" t="s">
         <v>21</v>
@@ -24625,7 +24629,7 @@
         <v>26</v>
       </c>
       <c r="G529" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H529" s="6" t="s">
         <v>21</v>
@@ -24666,7 +24670,7 @@
         <v>27</v>
       </c>
       <c r="G530" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H530" s="6" t="s">
         <v>21</v>
@@ -24707,7 +24711,7 @@
         <v>28</v>
       </c>
       <c r="G531" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H531" s="6" t="s">
         <v>21</v>
@@ -24801,7 +24805,7 @@
         <v>26</v>
       </c>
       <c r="G533" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H533" s="6" t="s">
         <v>21</v>
@@ -24842,7 +24846,7 @@
         <v>27</v>
       </c>
       <c r="G534" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H534" s="6" t="s">
         <v>21</v>
@@ -24883,7 +24887,7 @@
         <v>28</v>
       </c>
       <c r="G535" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H535" s="6" t="s">
         <v>21</v>
@@ -25030,7 +25034,7 @@
         <v>26</v>
       </c>
       <c r="G538" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="H538" s="6" t="s">
         <v>21</v>
@@ -25071,7 +25075,7 @@
         <v>27</v>
       </c>
       <c r="G539" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="H539" s="6" t="s">
         <v>21</v>
@@ -25112,7 +25116,7 @@
         <v>28</v>
       </c>
       <c r="G540" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="H540" s="6" t="s">
         <v>21</v>
@@ -25206,7 +25210,7 @@
         <v>26</v>
       </c>
       <c r="G542" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="H542" s="6" t="s">
         <v>21</v>
@@ -25247,7 +25251,7 @@
         <v>27</v>
       </c>
       <c r="G543" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="H543" s="6" t="s">
         <v>21</v>
@@ -25288,7 +25292,7 @@
         <v>28</v>
       </c>
       <c r="G544" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="H544" s="6" t="s">
         <v>21</v>
@@ -25382,7 +25386,7 @@
         <v>26</v>
       </c>
       <c r="G546" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="H546" s="6" t="s">
         <v>21</v>
@@ -25423,7 +25427,7 @@
         <v>27</v>
       </c>
       <c r="G547" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="H547" s="6" t="s">
         <v>21</v>
@@ -25464,7 +25468,7 @@
         <v>28</v>
       </c>
       <c r="G548" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="H548" s="6" t="s">
         <v>21</v>
@@ -25558,7 +25562,7 @@
         <v>26</v>
       </c>
       <c r="G550" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="H550" s="6" t="s">
         <v>21</v>
@@ -25599,7 +25603,7 @@
         <v>27</v>
       </c>
       <c r="G551" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="H551" s="6" t="s">
         <v>21</v>
@@ -25640,7 +25644,7 @@
         <v>28</v>
       </c>
       <c r="G552" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="H552" s="6" t="s">
         <v>21</v>
@@ -25686,8 +25690,10 @@
       <c r="C553" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="D553" s="6" t="s">
-        <v>80</v>
+      <c r="D553" s="6" t="inlineStr">
+        <is>
+          <t>Молот великанов</t>
+        </is>
       </c>
       <c r="E553" s="6">
         <v>25</v>
@@ -25734,7 +25740,7 @@
         <v>26</v>
       </c>
       <c r="G554" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="H554" s="6" t="s">
         <v>21</v>
@@ -25775,7 +25781,7 @@
         <v>27</v>
       </c>
       <c r="G555" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="H555" s="6" t="s">
         <v>21</v>
@@ -25816,7 +25822,7 @@
         <v>28</v>
       </c>
       <c r="G556" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="H556" s="6" t="s">
         <v>21</v>
@@ -25862,8 +25868,10 @@
       <c r="C557" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="D557" s="6" t="s">
-        <v>84</v>
+      <c r="D557" s="6" t="inlineStr">
+        <is>
+          <t>Громовой молот</t>
+        </is>
       </c>
       <c r="E557" s="6">
         <v>30</v>
@@ -25910,7 +25918,7 @@
         <v>26</v>
       </c>
       <c r="G558" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="H558" s="6" t="s">
         <v>21</v>
@@ -25951,7 +25959,7 @@
         <v>27</v>
       </c>
       <c r="G559" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="H559" s="6" t="s">
         <v>21</v>
@@ -25992,7 +26000,7 @@
         <v>28</v>
       </c>
       <c r="G560" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="H560" s="6" t="s">
         <v>21</v>
@@ -26086,7 +26094,7 @@
         <v>26</v>
       </c>
       <c r="G562" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="H562" s="6" t="s">
         <v>21</v>
@@ -26127,7 +26135,7 @@
         <v>27</v>
       </c>
       <c r="G563" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="H563" s="6" t="s">
         <v>21</v>
@@ -26168,7 +26176,7 @@
         <v>28</v>
       </c>
       <c r="G564" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="H564" s="6" t="s">
         <v>21</v>
@@ -26262,7 +26270,7 @@
         <v>26</v>
       </c>
       <c r="G566" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="H566" s="6" t="s">
         <v>21</v>
@@ -26303,7 +26311,7 @@
         <v>27</v>
       </c>
       <c r="G567" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="H567" s="6" t="s">
         <v>21</v>
@@ -26344,7 +26352,7 @@
         <v>28</v>
       </c>
       <c r="G568" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="H568" s="6" t="s">
         <v>21</v>
@@ -26438,7 +26446,7 @@
         <v>26</v>
       </c>
       <c r="G570" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="H570" s="6" t="s">
         <v>21</v>
@@ -26479,7 +26487,7 @@
         <v>27</v>
       </c>
       <c r="G571" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="H571" s="6" t="s">
         <v>21</v>
@@ -26520,7 +26528,7 @@
         <v>28</v>
       </c>
       <c r="G572" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="H572" s="6" t="s">
         <v>21</v>
@@ -26614,7 +26622,7 @@
         <v>26</v>
       </c>
       <c r="G574" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="H574" s="6" t="s">
         <v>21</v>
@@ -26655,7 +26663,7 @@
         <v>27</v>
       </c>
       <c r="G575" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="H575" s="6" t="s">
         <v>21</v>
@@ -26696,7 +26704,7 @@
         <v>28</v>
       </c>
       <c r="G576" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="H576" s="6" t="s">
         <v>21</v>
@@ -26849,7 +26857,7 @@
         <v>21</v>
       </c>
       <c r="I579" s="8">
-        <v>22.516710698714352</v>
+        <v>23</v>
       </c>
       <c r="J579" s="6" t="s">
         <v>21</v>
@@ -26890,7 +26898,7 @@
         <v>21</v>
       </c>
       <c r="I580" s="8">
-        <v>28.145888373392939</v>
+        <v>28</v>
       </c>
       <c r="J580" s="6" t="s">
         <v>21</v>
@@ -26931,7 +26939,7 @@
         <v>21</v>
       </c>
       <c r="I581" s="8">
-        <v>35.182360466741173</v>
+        <v>35</v>
       </c>
       <c r="J581" s="6" t="s">
         <v>21</v>
@@ -27025,7 +27033,7 @@
         <v>21</v>
       </c>
       <c r="I583" s="8">
-        <v>49.967709605353768</v>
+        <v>50</v>
       </c>
       <c r="J583" s="6" t="s">
         <v>21</v>
@@ -27066,7 +27074,7 @@
         <v>21</v>
       </c>
       <c r="I584" s="8">
-        <v>62.459637006692212</v>
+        <v>62</v>
       </c>
       <c r="J584" s="6" t="s">
         <v>21</v>
@@ -27107,7 +27115,7 @@
         <v>21</v>
       </c>
       <c r="I585" s="8">
-        <v>78.07454625836526</v>
+        <v>78</v>
       </c>
       <c r="J585" s="6" t="s">
         <v>21</v>
@@ -27201,7 +27209,7 @@
         <v>21</v>
       </c>
       <c r="I587" s="8">
-        <v>79.651579226632379</v>
+        <v>80</v>
       </c>
       <c r="J587" s="6" t="s">
         <v>21</v>
@@ -27242,7 +27250,7 @@
         <v>21</v>
       </c>
       <c r="I588" s="8">
-        <v>99.56447403329048</v>
+        <v>100</v>
       </c>
       <c r="J588" s="6" t="s">
         <v>21</v>
@@ -27283,7 +27291,7 @@
         <v>21</v>
       </c>
       <c r="I589" s="8">
-        <v>124.4555925416131</v>
+        <v>124</v>
       </c>
       <c r="J589" s="6" t="s">
         <v>21</v>
@@ -27377,7 +27385,7 @@
         <v>21</v>
       </c>
       <c r="I591" s="8">
-        <v>110.88529033450349</v>
+        <v>111</v>
       </c>
       <c r="J591" s="6" t="s">
         <v>21</v>
@@ -27418,7 +27426,7 @@
         <v>21</v>
       </c>
       <c r="I592" s="8">
-        <v>138.60661291812937</v>
+        <v>139</v>
       </c>
       <c r="J592" s="6" t="s">
         <v>21</v>
@@ -27459,7 +27467,7 @@
         <v>21</v>
       </c>
       <c r="I593" s="8">
-        <v>173.25826614766171</v>
+        <v>173</v>
       </c>
       <c r="J593" s="6" t="s">
         <v>21</v>
@@ -27553,7 +27561,7 @@
         <v>21</v>
       </c>
       <c r="I595" s="8">
-        <v>143.32450578361843</v>
+        <v>143</v>
       </c>
       <c r="J595" s="6" t="s">
         <v>21</v>
@@ -27594,7 +27602,7 @@
         <v>21</v>
       </c>
       <c r="I596" s="8">
-        <v>179.15563222952304</v>
+        <v>179</v>
       </c>
       <c r="J596" s="6" t="s">
         <v>21</v>
@@ -27635,7 +27643,7 @@
         <v>21</v>
       </c>
       <c r="I597" s="8">
-        <v>223.94454028690379</v>
+        <v>224</v>
       </c>
       <c r="J597" s="6" t="s">
         <v>21</v>
@@ -27729,7 +27737,7 @@
         <v>21</v>
       </c>
       <c r="I599" s="8">
-        <v>176.75792142372919</v>
+        <v>177</v>
       </c>
       <c r="J599" s="6" t="s">
         <v>21</v>
@@ -27770,7 +27778,7 @@
         <v>21</v>
       </c>
       <c r="I600" s="8">
-        <v>220.94740177966148</v>
+        <v>221</v>
       </c>
       <c r="J600" s="6" t="s">
         <v>21</v>
@@ -27811,7 +27819,7 @@
         <v>21</v>
       </c>
       <c r="I601" s="8">
-        <v>276.18425222457682</v>
+        <v>276</v>
       </c>
       <c r="J601" s="6" t="s">
         <v>21</v>
@@ -27905,7 +27913,7 @@
         <v>21</v>
       </c>
       <c r="I603" s="8">
-        <v>211.04141686656769</v>
+        <v>211</v>
       </c>
       <c r="J603" s="6" t="s">
         <v>21</v>
@@ -27946,7 +27954,7 @@
         <v>21</v>
       </c>
       <c r="I604" s="8">
-        <v>263.80177108320959</v>
+        <v>264</v>
       </c>
       <c r="J604" s="6" t="s">
         <v>21</v>
@@ -27987,7 +27995,7 @@
         <v>21</v>
       </c>
       <c r="I605" s="8">
-        <v>329.75221385401198</v>
+        <v>330</v>
       </c>
       <c r="J605" s="6" t="s">
         <v>21</v>
@@ -28081,7 +28089,7 @@
         <v>21</v>
       </c>
       <c r="I607" s="8">
-        <v>246.06986611308943</v>
+        <v>246</v>
       </c>
       <c r="J607" s="6" t="s">
         <v>21</v>
@@ -28122,7 +28130,7 @@
         <v>21</v>
       </c>
       <c r="I608" s="8">
-        <v>307.5873326413618</v>
+        <v>308</v>
       </c>
       <c r="J608" s="6" t="s">
         <v>21</v>
@@ -28163,7 +28171,7 @@
         <v>21</v>
       </c>
       <c r="I609" s="8">
-        <v>384.48416580170226</v>
+        <v>384</v>
       </c>
       <c r="J609" s="6" t="s">
         <v>21</v>
@@ -28257,7 +28265,7 @@
         <v>21</v>
       </c>
       <c r="I611" s="8">
-        <v>281.7629163596593</v>
+        <v>282</v>
       </c>
       <c r="J611" s="6" t="s">
         <v>21</v>
@@ -28298,7 +28306,7 @@
         <v>21</v>
       </c>
       <c r="I612" s="8">
-        <v>352.20364544957414</v>
+        <v>352</v>
       </c>
       <c r="J612" s="6" t="s">
         <v>21</v>
@@ -28339,7 +28347,7 @@
         <v>21</v>
       </c>
       <c r="I613" s="8">
-        <v>440.25455681196769</v>
+        <v>440</v>
       </c>
       <c r="J613" s="6" t="s">
         <v>21</v>
@@ -28433,7 +28441,7 @@
         <v>21</v>
       </c>
       <c r="I615" s="8">
-        <v>318.05699243342849</v>
+        <v>318</v>
       </c>
       <c r="J615" s="6" t="s">
         <v>21</v>
@@ -28474,7 +28482,7 @@
         <v>21</v>
       </c>
       <c r="I616" s="8">
-        <v>397.57124054178564</v>
+        <v>398</v>
       </c>
       <c r="J616" s="6" t="s">
         <v>21</v>
@@ -28515,7 +28523,7 @@
         <v>21</v>
       </c>
       <c r="I617" s="8">
-        <v>496.96405067723208</v>
+        <v>497</v>
       </c>
       <c r="J617" s="6" t="s">
         <v>21</v>

</xml_diff>